<commit_message>
resumen rev total estudiantes
</commit_message>
<xml_diff>
--- a/backend/templates/Resumen_3ro.xlsx
+++ b/backend/templates/Resumen_3ro.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JavierWorkSpace\BatallaProject\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C097972-8337-4AF2-BF01-61BFC92A6367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CB6702-D547-4907-BE10-EC5D4CEC58C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{299BAFB4-AE58-4015-B36E-D7CD92F1B4DD}"/>
   </bookViews>
@@ -399,6 +399,7 @@
     <definedName name="inst_grade">'3er Año'!$P$62</definedName>
     <definedName name="inst_level">'3er Año'!$P$58</definedName>
     <definedName name="inst_municipality">'3er Año'!$C$9</definedName>
+    <definedName name="inst_name">'3er Año'!$J$7</definedName>
     <definedName name="inst_period">'3er Año'!$M$3</definedName>
     <definedName name="inst_phone">'3er Año'!$U$8</definedName>
     <definedName name="inst_section">'3er Año'!$P$65</definedName>
@@ -2819,22 +2820,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>59556</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>9861</xdr:rowOff>
+      <xdr:colOff>32845</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>55842</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>938237</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>180639</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>373664</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>26274</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9AF1E56B-9219-4254-B7DE-B5A2CFE036C5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{728BCFD8-210D-4DDE-92AA-973B049A6DE5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2843,20 +2844,15 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="59556" y="134419"/>
-          <a:ext cx="4593431" cy="690989"/>
+          <a:off x="32845" y="55842"/>
+          <a:ext cx="3465019" cy="818157"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3558,7 +3554,7 @@
       <c r="Y12" s="223"/>
       <c r="Z12" s="224"/>
     </row>
-    <row r="13" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:28" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="78"/>
       <c r="B13" s="82"/>
       <c r="C13" s="83"/>
@@ -6908,7 +6904,7 @@
       <c r="Y68" s="200"/>
       <c r="Z68" s="201"/>
     </row>
-    <row r="69" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="192" t="s">
         <v>69</v>
       </c>
@@ -6944,7 +6940,7 @@
       <c r="Y69" s="137"/>
       <c r="Z69" s="202"/>
     </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="192" t="s">
         <v>70</v>
       </c>
@@ -6976,7 +6972,7 @@
       <c r="Y70" s="203"/>
       <c r="Z70" s="204"/>
     </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="192" t="s">
         <v>71</v>
       </c>
@@ -7006,7 +7002,7 @@
       <c r="Y71" s="203"/>
       <c r="Z71" s="204"/>
     </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="188"/>
       <c r="B72" s="189"/>
       <c r="C72" s="189"/>
@@ -7036,7 +7032,7 @@
       <c r="Y72" s="203"/>
       <c r="Z72" s="204"/>
     </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="192" t="s">
         <v>72</v>
       </c>
@@ -7066,7 +7062,7 @@
       <c r="Y73" s="203"/>
       <c r="Z73" s="204"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="195"/>
       <c r="B74" s="63"/>
       <c r="C74" s="63"/>
@@ -7096,7 +7092,7 @@
       <c r="Y74" s="203"/>
       <c r="Z74" s="204"/>
     </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:26" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="170" t="s">
         <v>73</v>
       </c>
@@ -7126,7 +7122,7 @@
       <c r="Y75" s="203"/>
       <c r="Z75" s="204"/>
     </row>
-    <row r="76" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:26" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="176"/>
       <c r="B76" s="177"/>
       <c r="C76" s="177"/>
@@ -7419,8 +7415,8 @@
     <mergeCell ref="N4:V4"/>
     <mergeCell ref="A6:D6"/>
   </mergeCells>
-  <pageMargins left="0.1" right="0" top="0.1" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="14" scale="74" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.3" right="0.25" top="0.3" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="14" scale="71" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>